<commit_message>
evaluation: complete week3 RAG chat assessment
</commit_message>
<xml_diff>
--- a/eval/day4_results(Optimized-v2).xlsx
+++ b/eval/day4_results(Optimized-v2).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ragflow-maxkb-support\eval\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30E64CDB-AF23-4845-A6AF-7CC2503950DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{869987B2-88E6-4CA7-84CF-6465A2A0F7AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2600" yWindow="8280" windowWidth="34490" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9650" yWindow="6470" windowWidth="17990" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -159,9 +159,6 @@
     <t>如何配置模型？</t>
   </si>
   <si>
-    <t>model_summary.md / model_param.md / quick_start.md</t>
-  </si>
-  <si>
     <t>Q15</t>
   </si>
   <si>
@@ -242,6 +239,10 @@
   </si>
   <si>
     <t>如何上传并解析知识库文档？</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>model_summary.md / model_param.md / quick_start.md</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -591,7 +592,7 @@
     <col min="7" max="7" width="8.6640625" style="1"/>
     <col min="8" max="8" width="18.25" style="1" customWidth="1"/>
     <col min="9" max="9" width="23.08203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="14.08203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="16.9140625" style="1" customWidth="1"/>
     <col min="11" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
@@ -638,7 +639,7 @@
         <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>13</v>
@@ -670,7 +671,7 @@
         <v>12</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>15</v>
@@ -713,7 +714,7 @@
         <v>12</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>19</v>
@@ -745,7 +746,7 @@
         <v>12</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>21</v>
@@ -777,7 +778,7 @@
         <v>23</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>24</v>
@@ -791,7 +792,7 @@
         <v>23</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>26</v>
@@ -845,7 +846,7 @@
         <v>23</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>32</v>
@@ -941,7 +942,7 @@
         <v>34</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>41</v>
@@ -976,7 +977,7 @@
         <v>43</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="E15" s="1">
         <v>1</v>
@@ -999,16 +1000,16 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="D16" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>48</v>
       </c>
       <c r="E16" s="1">
         <v>1</v>
@@ -1031,16 +1032,16 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>50</v>
-      </c>
       <c r="D17" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E17" s="1">
         <v>1</v>
@@ -1063,16 +1064,16 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18" s="1" t="s">
+      <c r="D18" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="E18" s="1">
         <v>1</v>
@@ -1095,16 +1096,16 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="D19" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E19" s="1">
         <v>1</v>
@@ -1127,13 +1128,13 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="E20" s="1">
         <v>0</v>
@@ -1142,18 +1143,18 @@
         <v>0</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="E21" s="1">
         <v>0</v>
@@ -1162,7 +1163,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>